<commit_message>
Add sample output and README with terminal screenshot
</commit_message>
<xml_diff>
--- a/output/CRE_Model_Output.xlsx
+++ b/output/CRE_Model_Output.xlsx
@@ -7,9 +7,10 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Asset" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Rent_Roll" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Pro_Forma" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Asset" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Rent_Roll" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Pro_Forma" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -415,6 +416,92 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:B7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Metric</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Dataset Records</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>307919</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Office Assets</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>15907</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Building Size (SF)</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>50000</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Year 1 NOI</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>901700</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Annual Debt Service</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>250250</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Year 1 DSCR</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>3.603196803196803</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:DM2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
@@ -1343,7 +1430,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1460,13 +1547,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H6"/>
+  <dimension ref="A1:I6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1510,6 +1597,11 @@
           <t>CoC_Return</t>
         </is>
       </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>DSCR</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -1536,6 +1628,9 @@
       <c r="H2" t="n">
         <v>0.3948181818181818</v>
       </c>
+      <c r="I2" t="n">
+        <v>3.603196803196803</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -1562,6 +1657,9 @@
       <c r="H3" t="n">
         <v>0.4120006060606061</v>
       </c>
+      <c r="I3" t="n">
+        <v>3.716487512487512</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -1588,6 +1686,9 @@
       <c r="H4" t="n">
         <v>0.4297142606060605</v>
       </c>
+      <c r="I4" t="n">
+        <v>3.833280839160838</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -1614,6 +1715,9 @@
       <c r="H5" t="n">
         <v>0.4479753975151516</v>
       </c>
+      <c r="I5" t="n">
+        <v>3.95368393966034</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -1639,6 +1743,9 @@
       </c>
       <c r="H6" t="n">
         <v>0.4668007627133334</v>
+      </c>
+      <c r="I6" t="n">
+        <v>4.077807226681319</v>
       </c>
     </row>
   </sheetData>

</xml_diff>